<commit_message>
EGTX.ST CR:c|high|misclassified. + Excel
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/EGTX.ST.xlsx
+++ b/data/stx_xlsx/EGTX.ST.xlsx
@@ -855,7 +855,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="[&gt;=100]#,###0.0\%;[&lt;=-100]-#,###0.0\%;#,###0.0\%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -898,6 +898,12 @@
     <font>
       <sz val="10.0"/>
       <color rgb="FFF5475B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10.0"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -969,7 +975,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1036,16 +1042,19 @@
     <xf borderId="3" fillId="0" fontId="7" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="3" fillId="0" fontId="8" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="7" numFmtId="3" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="8" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="3" fillId="0" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="8" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="3" fillId="0" fontId="9" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="7" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -2057,15 +2066,42 @@
       <c r="C33" s="20">
         <v>107.39</v>
       </c>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
+      <c r="D33" s="22">
+        <f t="shared" ref="D33:L33" si="1">SUM(D34:D36)</f>
+        <v>172.57</v>
+      </c>
+      <c r="E33" s="22">
+        <f t="shared" si="1"/>
+        <v>73.17</v>
+      </c>
+      <c r="F33" s="22">
+        <f t="shared" si="1"/>
+        <v>47.21</v>
+      </c>
+      <c r="G33" s="22">
+        <f t="shared" si="1"/>
+        <v>33.31</v>
+      </c>
+      <c r="H33" s="22">
+        <f t="shared" si="1"/>
+        <v>34.17</v>
+      </c>
+      <c r="I33" s="22">
+        <f t="shared" si="1"/>
+        <v>29.37</v>
+      </c>
+      <c r="J33" s="22">
+        <f t="shared" si="1"/>
+        <v>25.68</v>
+      </c>
+      <c r="K33" s="22">
+        <f t="shared" si="1"/>
+        <v>19.16</v>
+      </c>
+      <c r="L33" s="22">
+        <f t="shared" si="1"/>
+        <v>17.39</v>
+      </c>
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
@@ -2261,28 +2297,28 @@
       <c r="A41" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B41" s="22">
+      <c r="B41" s="23">
         <v>373.25</v>
       </c>
-      <c r="C41" s="22">
+      <c r="C41" s="23">
         <v>370.09</v>
       </c>
-      <c r="D41" s="22">
+      <c r="D41" s="23">
         <v>380.69</v>
       </c>
-      <c r="E41" s="22">
+      <c r="E41" s="23">
         <v>209.7</v>
       </c>
-      <c r="F41" s="22">
+      <c r="F41" s="23">
         <v>144.54</v>
       </c>
-      <c r="G41" s="22">
+      <c r="G41" s="23">
         <v>223.08</v>
       </c>
-      <c r="H41" s="22">
+      <c r="H41" s="23">
         <v>138.88</v>
       </c>
-      <c r="I41" s="22">
+      <c r="I41" s="23">
         <v>113.06</v>
       </c>
       <c r="J41" s="18">
@@ -2312,11 +2348,11 @@
       <c r="H42" s="16">
         <v>0.0</v>
       </c>
-      <c r="I42" s="23">
+      <c r="I42" s="24">
         <v>0.0</v>
       </c>
       <c r="J42" s="16"/>
-      <c r="K42" s="23">
+      <c r="K42" s="24">
         <v>0.0</v>
       </c>
       <c r="L42" s="16"/>
@@ -2325,37 +2361,37 @@
       <c r="A43" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="B43" s="24">
+      <c r="B43" s="25">
         <v>-360.01</v>
       </c>
-      <c r="C43" s="24">
+      <c r="C43" s="25">
         <v>-335.0</v>
       </c>
-      <c r="D43" s="24">
+      <c r="D43" s="25">
         <v>-323.27</v>
       </c>
-      <c r="E43" s="24">
+      <c r="E43" s="25">
         <v>-188.22</v>
       </c>
-      <c r="F43" s="24">
+      <c r="F43" s="25">
         <v>-105.91</v>
       </c>
-      <c r="G43" s="24">
+      <c r="G43" s="25">
         <v>-181.46</v>
       </c>
-      <c r="H43" s="25">
+      <c r="H43" s="26">
         <v>-62.05</v>
       </c>
-      <c r="I43" s="25">
+      <c r="I43" s="26">
         <v>-86.64</v>
       </c>
-      <c r="J43" s="25">
+      <c r="J43" s="26">
         <v>-85.31</v>
       </c>
-      <c r="K43" s="25">
+      <c r="K43" s="26">
         <v>-37.67</v>
       </c>
-      <c r="L43" s="25">
+      <c r="L43" s="26">
         <v>-42.1</v>
       </c>
     </row>
@@ -2500,7 +2536,7 @@
       <c r="H48" s="21">
         <v>-0.01</v>
       </c>
-      <c r="I48" s="23">
+      <c r="I48" s="24">
         <v>0.0</v>
       </c>
       <c r="J48" s="16">
@@ -2523,7 +2559,7 @@
       <c r="E49" s="16"/>
       <c r="F49" s="16"/>
       <c r="G49" s="16"/>
-      <c r="H49" s="23">
+      <c r="H49" s="24">
         <v>0.0</v>
       </c>
       <c r="I49" s="16"/>
@@ -2548,10 +2584,10 @@
       <c r="F50" s="21">
         <v>-0.19</v>
       </c>
-      <c r="G50" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="H50" s="23">
+      <c r="G50" s="24">
+        <v>0.0</v>
+      </c>
+      <c r="H50" s="24">
         <v>0.0</v>
       </c>
       <c r="I50" s="16"/>
@@ -2665,13 +2701,13 @@
       <c r="A56" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="B56" s="25">
+      <c r="B56" s="26">
         <v>-2.22</v>
       </c>
-      <c r="C56" s="25">
+      <c r="C56" s="26">
         <v>-14.03</v>
       </c>
-      <c r="D56" s="25">
+      <c r="D56" s="26">
         <v>-1.99</v>
       </c>
       <c r="E56" s="18">
@@ -2680,7 +2716,7 @@
       <c r="F56" s="18">
         <v>1.14</v>
       </c>
-      <c r="G56" s="25">
+      <c r="G56" s="26">
         <v>-0.74</v>
       </c>
       <c r="H56" s="18">
@@ -2715,11 +2751,11 @@
       <c r="I57" s="16">
         <v>0.0</v>
       </c>
-      <c r="J57" s="23">
+      <c r="J57" s="24">
         <v>0.0</v>
       </c>
       <c r="K57" s="16"/>
-      <c r="L57" s="23">
+      <c r="L57" s="24">
         <v>0.0</v>
       </c>
     </row>
@@ -2727,37 +2763,37 @@
       <c r="A58" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="B58" s="24">
+      <c r="B58" s="25">
         <v>-362.34</v>
       </c>
-      <c r="C58" s="24">
+      <c r="C58" s="25">
         <v>-349.03</v>
       </c>
-      <c r="D58" s="24">
+      <c r="D58" s="25">
         <v>-325.26</v>
       </c>
-      <c r="E58" s="24">
+      <c r="E58" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F58" s="24">
+      <c r="F58" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G58" s="24">
+      <c r="G58" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H58" s="25">
+      <c r="H58" s="26">
         <v>-57.16</v>
       </c>
-      <c r="I58" s="25">
+      <c r="I58" s="26">
         <v>-79.6</v>
       </c>
-      <c r="J58" s="25">
+      <c r="J58" s="26">
         <v>-85.15</v>
       </c>
-      <c r="K58" s="25">
+      <c r="K58" s="26">
         <v>-37.53</v>
       </c>
-      <c r="L58" s="25">
+      <c r="L58" s="26">
         <v>-41.91</v>
       </c>
     </row>
@@ -2807,7 +2843,7 @@
       <c r="C60" s="18">
         <v>0.31</v>
       </c>
-      <c r="D60" s="25">
+      <c r="D60" s="26">
         <v>-0.1</v>
       </c>
       <c r="E60" s="19">
@@ -2837,37 +2873,37 @@
       <c r="A61" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="B61" s="24">
+      <c r="B61" s="25">
         <v>-362.76</v>
       </c>
-      <c r="C61" s="24">
+      <c r="C61" s="25">
         <v>-349.34</v>
       </c>
-      <c r="D61" s="24">
+      <c r="D61" s="25">
         <v>-325.16</v>
       </c>
-      <c r="E61" s="24">
+      <c r="E61" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F61" s="24">
+      <c r="F61" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G61" s="24">
+      <c r="G61" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H61" s="25">
+      <c r="H61" s="26">
         <v>-57.16</v>
       </c>
-      <c r="I61" s="25">
+      <c r="I61" s="26">
         <v>-79.6</v>
       </c>
-      <c r="J61" s="25">
+      <c r="J61" s="26">
         <v>-85.15</v>
       </c>
-      <c r="K61" s="25">
+      <c r="K61" s="26">
         <v>-37.53</v>
       </c>
-      <c r="L61" s="25">
+      <c r="L61" s="26">
         <v>-41.91</v>
       </c>
     </row>
@@ -2875,37 +2911,37 @@
       <c r="A62" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="B62" s="24">
+      <c r="B62" s="25">
         <v>-362.76</v>
       </c>
-      <c r="C62" s="24">
+      <c r="C62" s="25">
         <v>-349.34</v>
       </c>
-      <c r="D62" s="24">
+      <c r="D62" s="25">
         <v>-325.16</v>
       </c>
-      <c r="E62" s="24">
+      <c r="E62" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F62" s="24">
+      <c r="F62" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G62" s="24">
+      <c r="G62" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H62" s="25">
+      <c r="H62" s="26">
         <v>-57.16</v>
       </c>
-      <c r="I62" s="25">
+      <c r="I62" s="26">
         <v>-79.6</v>
       </c>
-      <c r="J62" s="25">
+      <c r="J62" s="26">
         <v>-85.15</v>
       </c>
-      <c r="K62" s="25">
+      <c r="K62" s="26">
         <v>-37.53</v>
       </c>
-      <c r="L62" s="25">
+      <c r="L62" s="26">
         <v>-41.91</v>
       </c>
     </row>
@@ -2913,37 +2949,37 @@
       <c r="A63" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="B63" s="24">
+      <c r="B63" s="25">
         <v>-362.76</v>
       </c>
-      <c r="C63" s="24">
+      <c r="C63" s="25">
         <v>-349.34</v>
       </c>
-      <c r="D63" s="24">
+      <c r="D63" s="25">
         <v>-325.16</v>
       </c>
-      <c r="E63" s="24">
+      <c r="E63" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F63" s="24">
+      <c r="F63" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G63" s="24">
+      <c r="G63" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H63" s="25">
+      <c r="H63" s="26">
         <v>-57.16</v>
       </c>
-      <c r="I63" s="25">
+      <c r="I63" s="26">
         <v>-79.6</v>
       </c>
-      <c r="J63" s="25">
+      <c r="J63" s="26">
         <v>-85.15</v>
       </c>
-      <c r="K63" s="25">
+      <c r="K63" s="26">
         <v>-37.53</v>
       </c>
-      <c r="L63" s="25">
+      <c r="L63" s="26">
         <v>-41.91</v>
       </c>
     </row>
@@ -2951,37 +2987,37 @@
       <c r="A64" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="B64" s="24">
+      <c r="B64" s="25">
         <v>-362.76</v>
       </c>
-      <c r="C64" s="24">
+      <c r="C64" s="25">
         <v>-349.34</v>
       </c>
-      <c r="D64" s="24">
+      <c r="D64" s="25">
         <v>-325.16</v>
       </c>
-      <c r="E64" s="24">
+      <c r="E64" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F64" s="24">
+      <c r="F64" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G64" s="24">
+      <c r="G64" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H64" s="25">
+      <c r="H64" s="26">
         <v>-57.16</v>
       </c>
-      <c r="I64" s="25">
+      <c r="I64" s="26">
         <v>-79.6</v>
       </c>
-      <c r="J64" s="25">
+      <c r="J64" s="26">
         <v>-85.15</v>
       </c>
-      <c r="K64" s="25">
+      <c r="K64" s="26">
         <v>-37.53</v>
       </c>
-      <c r="L64" s="25">
+      <c r="L64" s="26">
         <v>-41.91</v>
       </c>
     </row>
@@ -3009,37 +3045,37 @@
       <c r="A66" s="17" t="s">
         <v>94</v>
       </c>
-      <c r="B66" s="24">
+      <c r="B66" s="25">
         <v>-362.76</v>
       </c>
-      <c r="C66" s="24">
+      <c r="C66" s="25">
         <v>-349.44</v>
       </c>
-      <c r="D66" s="24">
+      <c r="D66" s="25">
         <v>-325.36</v>
       </c>
-      <c r="E66" s="24">
+      <c r="E66" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F66" s="24">
+      <c r="F66" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G66" s="24">
+      <c r="G66" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H66" s="25">
+      <c r="H66" s="26">
         <v>-57.16</v>
       </c>
-      <c r="I66" s="25">
+      <c r="I66" s="26">
         <v>-79.6</v>
       </c>
-      <c r="J66" s="25">
+      <c r="J66" s="26">
         <v>-85.15</v>
       </c>
-      <c r="K66" s="25">
+      <c r="K66" s="26">
         <v>-37.53</v>
       </c>
-      <c r="L66" s="25">
+      <c r="L66" s="26">
         <v>-41.91</v>
       </c>
     </row>
@@ -3047,22 +3083,22 @@
       <c r="A67" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="B67" s="26">
+      <c r="B67" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C67" s="26">
+      <c r="C67" s="27">
         <v>-349.44</v>
       </c>
-      <c r="D67" s="26">
+      <c r="D67" s="27">
         <v>-325.36</v>
       </c>
-      <c r="E67" s="26">
+      <c r="E67" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F67" s="26">
+      <c r="F67" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G67" s="26">
+      <c r="G67" s="27">
         <v>-182.2</v>
       </c>
       <c r="H67" s="21">
@@ -3121,7 +3157,7 @@
       <c r="C69" s="18">
         <v>0.1</v>
       </c>
-      <c r="D69" s="25">
+      <c r="D69" s="26">
         <v>-0.1</v>
       </c>
       <c r="E69" s="19">
@@ -3149,31 +3185,31 @@
       <c r="A70" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="B70" s="24">
+      <c r="B70" s="25">
         <v>-362.45</v>
       </c>
-      <c r="C70" s="24">
+      <c r="C70" s="25">
         <v>-349.34</v>
       </c>
-      <c r="D70" s="24">
+      <c r="D70" s="25">
         <v>-325.46</v>
       </c>
-      <c r="E70" s="24">
+      <c r="E70" s="25">
         <v>-184.14</v>
       </c>
-      <c r="F70" s="24">
+      <c r="F70" s="25">
         <v>-104.77</v>
       </c>
-      <c r="G70" s="24">
+      <c r="G70" s="25">
         <v>-182.2</v>
       </c>
-      <c r="H70" s="25">
+      <c r="H70" s="26">
         <v>-57.16</v>
       </c>
       <c r="I70" s="18">
         <v>79.6</v>
       </c>
-      <c r="J70" s="25">
+      <c r="J70" s="26">
         <v>-85.15</v>
       </c>
       <c r="K70" s="19"/>
@@ -3411,22 +3447,22 @@
       <c r="A77" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="B77" s="26">
+      <c r="B77" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C77" s="26">
+      <c r="C77" s="27">
         <v>-349.44</v>
       </c>
-      <c r="D77" s="26">
+      <c r="D77" s="27">
         <v>-325.36</v>
       </c>
-      <c r="E77" s="26">
+      <c r="E77" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F77" s="26">
+      <c r="F77" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G77" s="26">
+      <c r="G77" s="27">
         <v>-182.2</v>
       </c>
       <c r="H77" s="21">
@@ -3449,22 +3485,22 @@
       <c r="A78" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="B78" s="26">
+      <c r="B78" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C78" s="26">
+      <c r="C78" s="27">
         <v>-349.34</v>
       </c>
-      <c r="D78" s="26">
+      <c r="D78" s="27">
         <v>-325.16</v>
       </c>
-      <c r="E78" s="26">
+      <c r="E78" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F78" s="26">
+      <c r="F78" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G78" s="26">
+      <c r="G78" s="27">
         <v>-182.2</v>
       </c>
       <c r="H78" s="21">
@@ -4093,22 +4129,22 @@
       <c r="A99" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="B99" s="26">
+      <c r="B99" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C99" s="26">
+      <c r="C99" s="27">
         <v>-349.44</v>
       </c>
-      <c r="D99" s="26">
+      <c r="D99" s="27">
         <v>-325.36</v>
       </c>
-      <c r="E99" s="26">
+      <c r="E99" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F99" s="26">
+      <c r="F99" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G99" s="26">
+      <c r="G99" s="27">
         <v>-182.2</v>
       </c>
       <c r="H99" s="21">
@@ -4131,22 +4167,22 @@
       <c r="A100" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="B100" s="26">
+      <c r="B100" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C100" s="26">
+      <c r="C100" s="27">
         <v>-349.34</v>
       </c>
-      <c r="D100" s="26">
+      <c r="D100" s="27">
         <v>-325.16</v>
       </c>
-      <c r="E100" s="26">
+      <c r="E100" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F100" s="26">
+      <c r="F100" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G100" s="26">
+      <c r="G100" s="27">
         <v>-182.2</v>
       </c>
       <c r="H100" s="21">
@@ -4169,22 +4205,22 @@
       <c r="A101" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="B101" s="26">
+      <c r="B101" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C101" s="26">
+      <c r="C101" s="27">
         <v>-349.44</v>
       </c>
-      <c r="D101" s="26">
+      <c r="D101" s="27">
         <v>-325.36</v>
       </c>
-      <c r="E101" s="26">
+      <c r="E101" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F101" s="26">
+      <c r="F101" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G101" s="26">
+      <c r="G101" s="27">
         <v>-182.2</v>
       </c>
       <c r="H101" s="21">
@@ -4207,22 +4243,22 @@
       <c r="A102" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="B102" s="26">
+      <c r="B102" s="27">
         <v>-362.76</v>
       </c>
-      <c r="C102" s="26">
+      <c r="C102" s="27">
         <v>-349.34</v>
       </c>
-      <c r="D102" s="26">
+      <c r="D102" s="27">
         <v>-325.16</v>
       </c>
-      <c r="E102" s="26">
+      <c r="E102" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F102" s="26">
+      <c r="F102" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G102" s="26">
+      <c r="G102" s="27">
         <v>-182.2</v>
       </c>
       <c r="H102" s="21">
@@ -5813,7 +5849,7 @@
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
-      <c r="F27" s="23">
+      <c r="F27" s="24">
         <v>0.0</v>
       </c>
       <c r="G27" s="16">
@@ -5821,7 +5857,7 @@
       </c>
       <c r="H27" s="16"/>
       <c r="I27" s="16"/>
-      <c r="J27" s="23">
+      <c r="J27" s="24">
         <v>0.0</v>
       </c>
       <c r="K27" s="16"/>
@@ -5831,34 +5867,34 @@
       <c r="A28" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="B28" s="22">
+      <c r="B28" s="23">
         <v>277.3</v>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="23">
         <v>390.78</v>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="23">
         <v>348.24</v>
       </c>
-      <c r="E28" s="22">
+      <c r="E28" s="23">
         <v>138.74</v>
       </c>
-      <c r="F28" s="22">
+      <c r="F28" s="23">
         <v>148.97</v>
       </c>
-      <c r="G28" s="22">
+      <c r="G28" s="23">
         <v>313.13</v>
       </c>
-      <c r="H28" s="22">
+      <c r="H28" s="23">
         <v>253.12</v>
       </c>
-      <c r="I28" s="22">
+      <c r="I28" s="23">
         <v>236.19</v>
       </c>
-      <c r="J28" s="22">
+      <c r="J28" s="23">
         <v>315.57</v>
       </c>
-      <c r="K28" s="22">
+      <c r="K28" s="23">
         <v>376.19</v>
       </c>
       <c r="L28" s="18">
@@ -6026,7 +6062,7 @@
       <c r="F34" s="21">
         <v>-0.06</v>
       </c>
-      <c r="G34" s="23">
+      <c r="G34" s="24">
         <v>0.0</v>
       </c>
       <c r="H34" s="16"/>
@@ -6241,7 +6277,7 @@
       </c>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
-      <c r="F43" s="23">
+      <c r="F43" s="24">
         <v>0.0</v>
       </c>
       <c r="G43" s="16">
@@ -6285,22 +6321,22 @@
       <c r="A45" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="B45" s="22">
+      <c r="B45" s="23">
         <v>421.64</v>
       </c>
-      <c r="C45" s="22">
+      <c r="C45" s="23">
         <v>423.78</v>
       </c>
-      <c r="D45" s="22">
+      <c r="D45" s="23">
         <v>417.1</v>
       </c>
-      <c r="E45" s="22">
+      <c r="E45" s="23">
         <v>389.4</v>
       </c>
-      <c r="F45" s="22">
+      <c r="F45" s="23">
         <v>405.66</v>
       </c>
-      <c r="G45" s="22">
+      <c r="G45" s="23">
         <v>435.57</v>
       </c>
       <c r="H45" s="18">
@@ -6332,7 +6368,7 @@
       <c r="F46" s="16">
         <v>0.0</v>
       </c>
-      <c r="G46" s="23">
+      <c r="G46" s="24">
         <v>0.0</v>
       </c>
       <c r="H46" s="16"/>
@@ -6345,34 +6381,34 @@
       <c r="A47" s="17" t="s">
         <v>163</v>
       </c>
-      <c r="B47" s="22">
+      <c r="B47" s="23">
         <v>698.83</v>
       </c>
-      <c r="C47" s="22">
+      <c r="C47" s="23">
         <v>814.56</v>
       </c>
-      <c r="D47" s="22">
+      <c r="D47" s="23">
         <v>765.34</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E47" s="23">
         <v>528.14</v>
       </c>
-      <c r="F47" s="22">
+      <c r="F47" s="23">
         <v>554.63</v>
       </c>
-      <c r="G47" s="22">
+      <c r="G47" s="23">
         <v>748.69</v>
       </c>
-      <c r="H47" s="22">
+      <c r="H47" s="23">
         <v>253.24</v>
       </c>
-      <c r="I47" s="22">
+      <c r="I47" s="23">
         <v>236.19</v>
       </c>
-      <c r="J47" s="22">
+      <c r="J47" s="23">
         <v>315.57</v>
       </c>
-      <c r="K47" s="22">
+      <c r="K47" s="23">
         <v>376.19</v>
       </c>
       <c r="L47" s="18">
@@ -6605,7 +6641,7 @@
       <c r="G55" s="16"/>
       <c r="H55" s="16"/>
       <c r="I55" s="16"/>
-      <c r="J55" s="23">
+      <c r="J55" s="24">
         <v>0.0</v>
       </c>
       <c r="K55" s="16"/>
@@ -6615,13 +6651,13 @@
       <c r="A56" s="17" t="s">
         <v>172</v>
       </c>
-      <c r="B56" s="22">
+      <c r="B56" s="23">
         <v>263.42</v>
       </c>
-      <c r="C56" s="22">
+      <c r="C56" s="23">
         <v>209.94</v>
       </c>
-      <c r="D56" s="22">
+      <c r="D56" s="23">
         <v>104.6</v>
       </c>
       <c r="E56" s="18">
@@ -6795,7 +6831,7 @@
       <c r="C63" s="18">
         <v>97.87</v>
       </c>
-      <c r="D63" s="22">
+      <c r="D63" s="23">
         <v>111.55</v>
       </c>
       <c r="E63" s="18">
@@ -6819,13 +6855,13 @@
       <c r="A64" s="17" t="s">
         <v>179</v>
       </c>
-      <c r="B64" s="22">
+      <c r="B64" s="23">
         <v>328.48</v>
       </c>
-      <c r="C64" s="22">
+      <c r="C64" s="23">
         <v>307.81</v>
       </c>
-      <c r="D64" s="22">
+      <c r="D64" s="23">
         <v>216.15</v>
       </c>
       <c r="E64" s="18">
@@ -6961,34 +6997,34 @@
       <c r="A68" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="B68" s="26">
+      <c r="B68" s="27">
         <v>-2130.4</v>
       </c>
-      <c r="C68" s="26">
+      <c r="C68" s="27">
         <v>-1655.34</v>
       </c>
-      <c r="D68" s="26">
+      <c r="D68" s="27">
         <v>-1275.07</v>
       </c>
-      <c r="E68" s="26">
+      <c r="E68" s="27">
         <v>-884.41</v>
       </c>
-      <c r="F68" s="26">
+      <c r="F68" s="27">
         <v>-726.61</v>
       </c>
-      <c r="G68" s="26">
+      <c r="G68" s="27">
         <v>-669.59</v>
       </c>
-      <c r="H68" s="26">
+      <c r="H68" s="27">
         <v>-434.34</v>
       </c>
-      <c r="I68" s="26">
+      <c r="I68" s="27">
         <v>-392.1</v>
       </c>
-      <c r="J68" s="26">
+      <c r="J68" s="27">
         <v>-317.0</v>
       </c>
-      <c r="K68" s="26">
+      <c r="K68" s="27">
         <v>-217.03</v>
       </c>
       <c r="L68" s="21">
@@ -7023,34 +7059,34 @@
       <c r="A70" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="B70" s="22">
+      <c r="B70" s="23">
         <v>370.36</v>
       </c>
-      <c r="C70" s="22">
+      <c r="C70" s="23">
         <v>506.75</v>
       </c>
-      <c r="D70" s="22">
+      <c r="D70" s="23">
         <v>549.29</v>
       </c>
-      <c r="E70" s="22">
+      <c r="E70" s="23">
         <v>476.47</v>
       </c>
-      <c r="F70" s="22">
+      <c r="F70" s="23">
         <v>513.48</v>
       </c>
-      <c r="G70" s="22">
+      <c r="G70" s="23">
         <v>658.6</v>
       </c>
-      <c r="H70" s="22">
+      <c r="H70" s="23">
         <v>229.61</v>
       </c>
-      <c r="I70" s="22">
+      <c r="I70" s="23">
         <v>214.07</v>
       </c>
-      <c r="J70" s="22">
+      <c r="J70" s="23">
         <v>303.91</v>
       </c>
-      <c r="K70" s="22">
+      <c r="K70" s="23">
         <v>369.43</v>
       </c>
       <c r="L70" s="18">
@@ -7061,34 +7097,34 @@
       <c r="A71" s="17" t="s">
         <v>186</v>
       </c>
-      <c r="B71" s="22">
+      <c r="B71" s="23">
         <v>370.36</v>
       </c>
-      <c r="C71" s="22">
+      <c r="C71" s="23">
         <v>506.75</v>
       </c>
-      <c r="D71" s="22">
+      <c r="D71" s="23">
         <v>549.29</v>
       </c>
-      <c r="E71" s="22">
+      <c r="E71" s="23">
         <v>476.47</v>
       </c>
-      <c r="F71" s="22">
+      <c r="F71" s="23">
         <v>513.48</v>
       </c>
-      <c r="G71" s="22">
+      <c r="G71" s="23">
         <v>658.6</v>
       </c>
-      <c r="H71" s="22">
+      <c r="H71" s="23">
         <v>229.61</v>
       </c>
-      <c r="I71" s="22">
+      <c r="I71" s="23">
         <v>214.07</v>
       </c>
-      <c r="J71" s="22">
+      <c r="J71" s="23">
         <v>303.91</v>
       </c>
-      <c r="K71" s="22">
+      <c r="K71" s="23">
         <v>369.43</v>
       </c>
       <c r="L71" s="18">
@@ -7109,7 +7145,7 @@
       <c r="G72" s="16">
         <v>0.0</v>
       </c>
-      <c r="H72" s="23">
+      <c r="H72" s="24">
         <v>0.0</v>
       </c>
       <c r="I72" s="16"/>
@@ -7121,34 +7157,34 @@
       <c r="A73" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="B73" s="22">
+      <c r="B73" s="23">
         <v>698.83</v>
       </c>
-      <c r="C73" s="22">
+      <c r="C73" s="23">
         <v>814.56</v>
       </c>
-      <c r="D73" s="22">
+      <c r="D73" s="23">
         <v>765.34</v>
       </c>
-      <c r="E73" s="22">
+      <c r="E73" s="23">
         <v>528.14</v>
       </c>
-      <c r="F73" s="22">
+      <c r="F73" s="23">
         <v>554.63</v>
       </c>
-      <c r="G73" s="22">
+      <c r="G73" s="23">
         <v>748.69</v>
       </c>
-      <c r="H73" s="22">
+      <c r="H73" s="23">
         <v>253.24</v>
       </c>
-      <c r="I73" s="22">
+      <c r="I73" s="23">
         <v>236.19</v>
       </c>
-      <c r="J73" s="22">
+      <c r="J73" s="23">
         <v>315.57</v>
       </c>
-      <c r="K73" s="22">
+      <c r="K73" s="23">
         <v>376.19</v>
       </c>
       <c r="L73" s="18">
@@ -8882,962 +8918,962 @@
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="27" t="s">
+      <c r="A20" s="28" t="s">
         <v>215</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="28"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="28"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="28"/>
-      <c r="Q20" s="28"/>
-      <c r="R20" s="28"/>
-      <c r="S20" s="28"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
+      <c r="H20" s="29"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
+      <c r="K20" s="29"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="29"/>
+      <c r="P20" s="29"/>
+      <c r="Q20" s="29"/>
+      <c r="R20" s="29"/>
+      <c r="S20" s="29"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="30" t="s">
         <v>215</v>
       </c>
-      <c r="B21" s="30">
+      <c r="B21" s="31">
         <v>2344.85</v>
       </c>
-      <c r="C21" s="30">
+      <c r="C21" s="31">
         <v>1452.01</v>
       </c>
-      <c r="D21" s="30">
+      <c r="D21" s="31">
         <v>1316.44</v>
       </c>
-      <c r="E21" s="30">
+      <c r="E21" s="31">
         <v>942.9</v>
       </c>
-      <c r="F21" s="30">
+      <c r="F21" s="31">
         <v>991.86</v>
       </c>
-      <c r="G21" s="30">
+      <c r="G21" s="31">
         <v>764.83</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="31">
         <v>499.92</v>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="31">
         <v>581.44</v>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="31">
         <v>434.01</v>
       </c>
-      <c r="K21" s="30">
+      <c r="K21" s="31">
         <v>1358.56</v>
       </c>
-      <c r="L21" s="30">
+      <c r="L21" s="31">
         <v>583.37</v>
       </c>
-      <c r="M21" s="30">
+      <c r="M21" s="31">
         <v>259.23</v>
       </c>
-      <c r="N21" s="30">
+      <c r="N21" s="31">
         <v>101.32</v>
       </c>
-      <c r="O21" s="30">
+      <c r="O21" s="31">
         <v>102.39</v>
       </c>
-      <c r="P21" s="31"/>
-      <c r="Q21" s="31"/>
-      <c r="R21" s="31"/>
-      <c r="S21" s="31"/>
+      <c r="P21" s="32"/>
+      <c r="Q21" s="32"/>
+      <c r="R21" s="32"/>
+      <c r="S21" s="32"/>
     </row>
     <row r="22" ht="15.0" customHeight="1">
-      <c r="A22" s="29" t="s">
+      <c r="A22" s="30" t="s">
         <v>216</v>
       </c>
-      <c r="B22" s="30">
+      <c r="B22" s="31">
         <v>1447.41</v>
       </c>
-      <c r="C22" s="30">
+      <c r="C22" s="31">
         <v>1122.38</v>
       </c>
-      <c r="D22" s="30">
+      <c r="D22" s="31">
         <v>874.29</v>
       </c>
-      <c r="E22" s="30">
+      <c r="E22" s="31">
         <v>745.66</v>
       </c>
-      <c r="F22" s="30">
+      <c r="F22" s="31">
         <v>692.64</v>
       </c>
-      <c r="G22" s="30">
+      <c r="G22" s="31">
         <v>687.27</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="31">
         <v>674.86</v>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="31">
         <v>644.52</v>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="31">
         <v>523.06</v>
       </c>
-      <c r="K22" s="30">
+      <c r="K22" s="31">
         <v>506.15</v>
       </c>
-      <c r="L22" s="31"/>
-      <c r="M22" s="31"/>
-      <c r="N22" s="31"/>
-      <c r="O22" s="31"/>
-      <c r="P22" s="31"/>
-      <c r="Q22" s="31"/>
-      <c r="R22" s="31"/>
-      <c r="S22" s="31"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="32"/>
+      <c r="Q22" s="32"/>
+      <c r="R22" s="32"/>
+      <c r="S22" s="32"/>
     </row>
     <row r="23" ht="15.0" customHeight="1">
-      <c r="A23" s="27" t="s">
+      <c r="A23" s="28" t="s">
         <v>217</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="28"/>
-      <c r="L23" s="28"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="28"/>
-      <c r="O23" s="28"/>
-      <c r="P23" s="28"/>
-      <c r="Q23" s="28"/>
-      <c r="R23" s="28"/>
-      <c r="S23" s="28"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
+      <c r="G23" s="29"/>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="29"/>
+      <c r="N23" s="29"/>
+      <c r="O23" s="29"/>
+      <c r="P23" s="29"/>
+      <c r="Q23" s="29"/>
+      <c r="R23" s="29"/>
+      <c r="S23" s="29"/>
     </row>
     <row r="24" ht="15.0" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="30" t="s">
         <v>217</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="31">
         <v>2585.32</v>
       </c>
-      <c r="C24" s="30">
+      <c r="C24" s="31">
         <v>1643.59</v>
       </c>
-      <c r="D24" s="30">
+      <c r="D24" s="31">
         <v>1434.1</v>
       </c>
-      <c r="E24" s="30">
+      <c r="E24" s="31">
         <v>1079.12</v>
       </c>
-      <c r="F24" s="30">
+      <c r="F24" s="31">
         <v>1287.56</v>
       </c>
-      <c r="G24" s="30">
+      <c r="G24" s="31">
         <v>1003.92</v>
       </c>
-      <c r="H24" s="30">
+      <c r="H24" s="31">
         <v>724.25</v>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="31">
         <v>891.17</v>
       </c>
-      <c r="J24" s="30">
+      <c r="J24" s="31">
         <v>807.65</v>
       </c>
-      <c r="K24" s="30">
+      <c r="K24" s="31">
         <v>1411.26</v>
       </c>
-      <c r="L24" s="30">
+      <c r="L24" s="31">
         <v>679.26</v>
       </c>
-      <c r="M24" s="30">
+      <c r="M24" s="31">
         <v>305.96</v>
       </c>
-      <c r="N24" s="30">
+      <c r="N24" s="31">
         <v>151.66</v>
       </c>
-      <c r="O24" s="30">
+      <c r="O24" s="31">
         <v>180.96</v>
       </c>
-      <c r="P24" s="31"/>
-      <c r="Q24" s="31"/>
-      <c r="R24" s="31"/>
-      <c r="S24" s="31"/>
+      <c r="P24" s="32"/>
+      <c r="Q24" s="32"/>
+      <c r="R24" s="32"/>
+      <c r="S24" s="32"/>
     </row>
     <row r="25" ht="15.0" customHeight="1">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="B25" s="30">
+      <c r="B25" s="31">
         <v>1647.31</v>
       </c>
-      <c r="C25" s="30">
+      <c r="C25" s="31">
         <v>1322.38</v>
       </c>
-      <c r="D25" s="30">
+      <c r="D25" s="31">
         <v>1068.73</v>
       </c>
-      <c r="E25" s="30">
+      <c r="E25" s="31">
         <v>982.87</v>
       </c>
-      <c r="F25" s="30">
+      <c r="F25" s="31">
         <v>999.96</v>
       </c>
-      <c r="G25" s="30">
+      <c r="G25" s="31">
         <v>919.58</v>
       </c>
-      <c r="H25" s="30">
+      <c r="H25" s="31">
         <v>886.39</v>
       </c>
-      <c r="I25" s="30">
+      <c r="I25" s="31">
         <v>825.34</v>
       </c>
-      <c r="J25" s="30">
+      <c r="J25" s="31">
         <v>646.87</v>
       </c>
-      <c r="K25" s="30">
+      <c r="K25" s="31">
         <v>579.27</v>
       </c>
-      <c r="L25" s="31"/>
-      <c r="M25" s="31"/>
-      <c r="N25" s="31"/>
-      <c r="O25" s="31"/>
-      <c r="P25" s="31"/>
-      <c r="Q25" s="31"/>
-      <c r="R25" s="31"/>
-      <c r="S25" s="31"/>
+      <c r="L25" s="32"/>
+      <c r="M25" s="32"/>
+      <c r="N25" s="32"/>
+      <c r="O25" s="32"/>
+      <c r="P25" s="32"/>
+      <c r="Q25" s="32"/>
+      <c r="R25" s="32"/>
+      <c r="S25" s="32"/>
     </row>
     <row r="26" ht="15.0" customHeight="1">
-      <c r="A26" s="27" t="s">
+      <c r="A26" s="28" t="s">
         <v>219</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="28"/>
-      <c r="K26" s="28"/>
-      <c r="L26" s="28"/>
-      <c r="M26" s="28"/>
-      <c r="N26" s="28"/>
-      <c r="O26" s="28"/>
-      <c r="P26" s="28"/>
-      <c r="Q26" s="28"/>
-      <c r="R26" s="28"/>
-      <c r="S26" s="28"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="29"/>
+      <c r="F26" s="29"/>
+      <c r="G26" s="29"/>
+      <c r="H26" s="29"/>
+      <c r="I26" s="29"/>
+      <c r="J26" s="29"/>
+      <c r="K26" s="29"/>
+      <c r="L26" s="29"/>
+      <c r="M26" s="29"/>
+      <c r="N26" s="29"/>
+      <c r="O26" s="29"/>
+      <c r="P26" s="29"/>
+      <c r="Q26" s="29"/>
+      <c r="R26" s="29"/>
+      <c r="S26" s="29"/>
     </row>
     <row r="27" ht="15.0" customHeight="1">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="30" t="s">
         <v>220</v>
       </c>
-      <c r="B27" s="32">
+      <c r="B27" s="33">
         <v>7.2</v>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="33">
         <v>5.62</v>
       </c>
-      <c r="D27" s="32">
+      <c r="D27" s="33">
         <v>6.68</v>
       </c>
-      <c r="E27" s="32">
+      <c r="E27" s="33">
         <v>6.0</v>
       </c>
-      <c r="F27" s="32">
+      <c r="F27" s="33">
         <v>7.16</v>
       </c>
-      <c r="G27" s="32">
+      <c r="G27" s="33">
         <v>16.96</v>
       </c>
-      <c r="H27" s="32">
+      <c r="H27" s="33">
         <v>13.46</v>
       </c>
-      <c r="I27" s="32">
+      <c r="I27" s="33">
         <v>16.56</v>
       </c>
-      <c r="J27" s="32">
+      <c r="J27" s="33">
         <v>15.01</v>
       </c>
-      <c r="K27" s="32">
+      <c r="K27" s="33">
         <v>44.95</v>
       </c>
-      <c r="L27" s="32">
+      <c r="L27" s="33">
         <v>21.67</v>
       </c>
-      <c r="M27" s="32">
+      <c r="M27" s="33">
         <v>11.78</v>
       </c>
-      <c r="N27" s="32">
+      <c r="N27" s="33">
         <v>6.24</v>
       </c>
-      <c r="O27" s="32">
+      <c r="O27" s="33">
         <v>7.44</v>
       </c>
-      <c r="P27" s="31"/>
-      <c r="Q27" s="31"/>
-      <c r="R27" s="31"/>
-      <c r="S27" s="31"/>
+      <c r="P27" s="32"/>
+      <c r="Q27" s="32"/>
+      <c r="R27" s="32"/>
+      <c r="S27" s="32"/>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="30" t="s">
         <v>221</v>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="33">
         <v>6.72</v>
       </c>
-      <c r="C28" s="32">
+      <c r="C28" s="33">
         <v>8.81</v>
       </c>
-      <c r="D28" s="32">
+      <c r="D28" s="33">
         <v>9.79</v>
       </c>
-      <c r="E28" s="32">
+      <c r="E28" s="33">
         <v>11.97</v>
       </c>
-      <c r="F28" s="32">
+      <c r="F28" s="33">
         <v>14.85</v>
       </c>
-      <c r="G28" s="32">
+      <c r="G28" s="33">
         <v>20.1</v>
       </c>
-      <c r="H28" s="32">
+      <c r="H28" s="33">
         <v>21.8</v>
       </c>
-      <c r="I28" s="32">
+      <c r="I28" s="33">
         <v>22.1</v>
       </c>
-      <c r="J28" s="32">
+      <c r="J28" s="33">
         <v>19.19</v>
       </c>
-      <c r="K28" s="32">
+      <c r="K28" s="33">
         <v>19.66</v>
       </c>
-      <c r="L28" s="31"/>
-      <c r="M28" s="31"/>
-      <c r="N28" s="31"/>
-      <c r="O28" s="31"/>
-      <c r="P28" s="31"/>
-      <c r="Q28" s="31"/>
-      <c r="R28" s="31"/>
-      <c r="S28" s="31"/>
+      <c r="L28" s="32"/>
+      <c r="M28" s="32"/>
+      <c r="N28" s="32"/>
+      <c r="O28" s="32"/>
+      <c r="P28" s="32"/>
+      <c r="Q28" s="32"/>
+      <c r="R28" s="32"/>
+      <c r="S28" s="32"/>
     </row>
     <row r="29" ht="15.0" customHeight="1">
-      <c r="A29" s="27" t="s">
+      <c r="A29" s="28" t="s">
         <v>222</v>
       </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-      <c r="E29" s="28"/>
-      <c r="F29" s="28"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="28"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="28"/>
-      <c r="K29" s="28"/>
-      <c r="L29" s="28"/>
-      <c r="M29" s="28"/>
-      <c r="N29" s="28"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="28"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="28"/>
-      <c r="S29" s="28"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
+      <c r="H29" s="29"/>
+      <c r="I29" s="29"/>
+      <c r="J29" s="29"/>
+      <c r="K29" s="29"/>
+      <c r="L29" s="29"/>
+      <c r="M29" s="29"/>
+      <c r="N29" s="29"/>
+      <c r="O29" s="29"/>
+      <c r="P29" s="29"/>
+      <c r="Q29" s="29"/>
+      <c r="R29" s="29"/>
+      <c r="S29" s="29"/>
     </row>
     <row r="30" ht="15.0" customHeight="1">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="30" t="s">
         <v>223</v>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="34">
         <v>-10.62</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C30" s="34">
         <v>-19.43</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="34">
         <v>-12.58</v>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="34">
         <v>-11.76</v>
       </c>
-      <c r="F30" s="33">
+      <c r="F30" s="34">
         <v>-26.75</v>
       </c>
-      <c r="G30" s="34"/>
-      <c r="H30" s="33">
+      <c r="G30" s="35"/>
+      <c r="H30" s="34">
         <v>-11.05</v>
       </c>
-      <c r="I30" s="33">
+      <c r="I30" s="34">
         <v>-9.72</v>
       </c>
-      <c r="J30" s="33">
+      <c r="J30" s="34">
         <v>-6.94</v>
       </c>
-      <c r="K30" s="33">
+      <c r="K30" s="34">
         <v>-3.8</v>
       </c>
-      <c r="L30" s="33">
+      <c r="L30" s="34">
         <v>-7.31</v>
       </c>
-      <c r="M30" s="33">
+      <c r="M30" s="34">
         <v>-8.65</v>
       </c>
-      <c r="N30" s="33">
+      <c r="N30" s="34">
         <v>-18.04</v>
       </c>
-      <c r="O30" s="33">
+      <c r="O30" s="34">
         <v>-15.31</v>
       </c>
-      <c r="P30" s="34"/>
-      <c r="Q30" s="34"/>
-      <c r="R30" s="34"/>
-      <c r="S30" s="34"/>
+      <c r="P30" s="35"/>
+      <c r="Q30" s="35"/>
+      <c r="R30" s="35"/>
+      <c r="S30" s="35"/>
     </row>
     <row r="31" ht="15.0" customHeight="1">
-      <c r="A31" s="29" t="s">
+      <c r="A31" s="30" t="s">
         <v>224</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="34">
         <v>-16.15</v>
       </c>
-      <c r="C31" s="34"/>
-      <c r="D31" s="34"/>
-      <c r="E31" s="34"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="34"/>
-      <c r="H31" s="33">
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="34">
         <v>-6.72</v>
       </c>
-      <c r="I31" s="33">
+      <c r="I31" s="34">
         <v>-6.4</v>
       </c>
-      <c r="J31" s="33">
+      <c r="J31" s="34">
         <v>-6.7</v>
       </c>
-      <c r="K31" s="33">
+      <c r="K31" s="34">
         <v>-7.44</v>
       </c>
-      <c r="L31" s="34"/>
-      <c r="M31" s="34"/>
-      <c r="N31" s="34"/>
-      <c r="O31" s="34"/>
-      <c r="P31" s="34"/>
-      <c r="Q31" s="34"/>
-      <c r="R31" s="34"/>
-      <c r="S31" s="34"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
+      <c r="O31" s="35"/>
+      <c r="P31" s="35"/>
+      <c r="Q31" s="35"/>
+      <c r="R31" s="35"/>
+      <c r="S31" s="35"/>
     </row>
     <row r="32" ht="15.0" customHeight="1">
-      <c r="A32" s="27" t="s">
+      <c r="A32" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
-      <c r="N32" s="28"/>
-      <c r="O32" s="28"/>
-      <c r="P32" s="28"/>
-      <c r="Q32" s="28"/>
-      <c r="R32" s="28"/>
-      <c r="S32" s="28"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+      <c r="I32" s="29"/>
+      <c r="J32" s="29"/>
+      <c r="K32" s="29"/>
+      <c r="L32" s="29"/>
+      <c r="M32" s="29"/>
+      <c r="N32" s="29"/>
+      <c r="O32" s="29"/>
+      <c r="P32" s="29"/>
+      <c r="Q32" s="29"/>
+      <c r="R32" s="29"/>
+      <c r="S32" s="29"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="30" t="s">
         <v>226</v>
       </c>
-      <c r="B33" s="32">
+      <c r="B33" s="33">
         <v>5.1</v>
       </c>
-      <c r="C33" s="32">
+      <c r="C33" s="33">
         <v>2.99</v>
       </c>
-      <c r="D33" s="32">
+      <c r="D33" s="33">
         <v>3.01</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E33" s="33">
         <v>2.1</v>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="33">
         <v>1.96</v>
       </c>
-      <c r="G33" s="32">
+      <c r="G33" s="33">
         <v>4.37</v>
       </c>
-      <c r="H33" s="32">
+      <c r="H33" s="33">
         <v>3.38</v>
       </c>
-      <c r="I33" s="32">
+      <c r="I33" s="33">
         <v>2.93</v>
       </c>
-      <c r="J33" s="32">
+      <c r="J33" s="33">
         <v>2.19</v>
       </c>
-      <c r="K33" s="32">
+      <c r="K33" s="33">
         <v>28.07</v>
       </c>
-      <c r="L33" s="32">
+      <c r="L33" s="33">
         <v>7.82</v>
       </c>
-      <c r="M33" s="32">
+      <c r="M33" s="33">
         <v>6.91</v>
       </c>
-      <c r="N33" s="32">
+      <c r="N33" s="33">
         <v>3.28</v>
       </c>
-      <c r="O33" s="32">
+      <c r="O33" s="33">
         <v>2.38</v>
       </c>
-      <c r="P33" s="31"/>
-      <c r="Q33" s="31"/>
-      <c r="R33" s="31"/>
-      <c r="S33" s="31"/>
+      <c r="P33" s="32"/>
+      <c r="Q33" s="32"/>
+      <c r="R33" s="32"/>
+      <c r="S33" s="32"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="29" t="s">
+      <c r="A34" s="30" t="s">
         <v>227</v>
       </c>
-      <c r="B34" s="32">
+      <c r="B34" s="33">
         <v>2.72</v>
       </c>
-      <c r="C34" s="32">
+      <c r="C34" s="33">
         <v>2.96</v>
       </c>
-      <c r="D34" s="32">
+      <c r="D34" s="33">
         <v>3.06</v>
       </c>
-      <c r="E34" s="32">
+      <c r="E34" s="33">
         <v>3.03</v>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="33">
         <v>2.89</v>
       </c>
-      <c r="G34" s="32">
+      <c r="G34" s="33">
         <v>4.74</v>
       </c>
-      <c r="H34" s="32">
+      <c r="H34" s="33">
         <v>5.23</v>
       </c>
-      <c r="I34" s="32">
+      <c r="I34" s="33">
         <v>5.78</v>
       </c>
-      <c r="J34" s="32">
+      <c r="J34" s="33">
         <v>6.45</v>
       </c>
-      <c r="K34" s="32">
+      <c r="K34" s="33">
         <v>7.79</v>
       </c>
-      <c r="L34" s="31"/>
-      <c r="M34" s="31"/>
-      <c r="N34" s="31"/>
-      <c r="O34" s="31"/>
-      <c r="P34" s="31"/>
-      <c r="Q34" s="31"/>
-      <c r="R34" s="31"/>
-      <c r="S34" s="31"/>
+      <c r="L34" s="32"/>
+      <c r="M34" s="32"/>
+      <c r="N34" s="32"/>
+      <c r="O34" s="32"/>
+      <c r="P34" s="32"/>
+      <c r="Q34" s="32"/>
+      <c r="R34" s="32"/>
+      <c r="S34" s="32"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="27" t="s">
+      <c r="A35" s="28" t="s">
         <v>228</v>
       </c>
-      <c r="B35" s="28"/>
-      <c r="C35" s="28"/>
-      <c r="D35" s="28"/>
-      <c r="E35" s="28"/>
-      <c r="F35" s="28"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="28"/>
-      <c r="J35" s="28"/>
-      <c r="K35" s="28"/>
-      <c r="L35" s="28"/>
-      <c r="M35" s="28"/>
-      <c r="N35" s="28"/>
-      <c r="O35" s="28"/>
-      <c r="P35" s="28"/>
-      <c r="Q35" s="28"/>
-      <c r="R35" s="28"/>
-      <c r="S35" s="28"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="29"/>
+      <c r="F35" s="29"/>
+      <c r="G35" s="29"/>
+      <c r="H35" s="29"/>
+      <c r="I35" s="29"/>
+      <c r="J35" s="29"/>
+      <c r="K35" s="29"/>
+      <c r="L35" s="29"/>
+      <c r="M35" s="29"/>
+      <c r="N35" s="29"/>
+      <c r="O35" s="29"/>
+      <c r="P35" s="29"/>
+      <c r="Q35" s="29"/>
+      <c r="R35" s="29"/>
+      <c r="S35" s="29"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="30" t="s">
         <v>229</v>
       </c>
-      <c r="B36" s="32">
+      <c r="B36" s="33">
         <v>29.62</v>
       </c>
-      <c r="C36" s="32">
+      <c r="C36" s="33">
         <v>11.96</v>
       </c>
-      <c r="D36" s="32">
+      <c r="D36" s="33">
         <v>15.87</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="33">
         <v>9.57</v>
       </c>
-      <c r="F36" s="32">
+      <c r="F36" s="33">
         <v>5.65</v>
       </c>
-      <c r="G36" s="32">
+      <c r="G36" s="33">
         <v>4.37</v>
       </c>
-      <c r="H36" s="32">
+      <c r="H36" s="33">
         <v>3.38</v>
       </c>
-      <c r="I36" s="32">
+      <c r="I36" s="33">
         <v>2.93</v>
       </c>
-      <c r="J36" s="32">
+      <c r="J36" s="33">
         <v>2.19</v>
       </c>
-      <c r="K36" s="32">
+      <c r="K36" s="33">
         <v>28.07</v>
       </c>
-      <c r="L36" s="32">
+      <c r="L36" s="33">
         <v>7.82</v>
       </c>
-      <c r="M36" s="32">
+      <c r="M36" s="33">
         <v>6.91</v>
       </c>
-      <c r="N36" s="32">
+      <c r="N36" s="33">
         <v>3.28</v>
       </c>
-      <c r="O36" s="32">
+      <c r="O36" s="33">
         <v>2.38</v>
       </c>
-      <c r="P36" s="31"/>
-      <c r="Q36" s="31"/>
-      <c r="R36" s="31"/>
-      <c r="S36" s="31"/>
+      <c r="P36" s="32"/>
+      <c r="Q36" s="32"/>
+      <c r="R36" s="32"/>
+      <c r="S36" s="32"/>
     </row>
     <row r="37" ht="15.0" customHeight="1">
-      <c r="A37" s="29" t="s">
+      <c r="A37" s="30" t="s">
         <v>230</v>
       </c>
-      <c r="B37" s="32">
+      <c r="B37" s="33">
         <v>10.87</v>
       </c>
-      <c r="C37" s="32">
+      <c r="C37" s="33">
         <v>6.34</v>
       </c>
-      <c r="D37" s="32">
+      <c r="D37" s="33">
         <v>4.94</v>
       </c>
-      <c r="E37" s="32">
+      <c r="E37" s="33">
         <v>3.91</v>
       </c>
-      <c r="F37" s="32">
+      <c r="F37" s="33">
         <v>3.19</v>
       </c>
-      <c r="G37" s="32">
+      <c r="G37" s="33">
         <v>4.74</v>
       </c>
-      <c r="H37" s="32">
+      <c r="H37" s="33">
         <v>5.23</v>
       </c>
-      <c r="I37" s="32">
+      <c r="I37" s="33">
         <v>5.78</v>
       </c>
-      <c r="J37" s="32">
+      <c r="J37" s="33">
         <v>6.45</v>
       </c>
-      <c r="K37" s="32">
+      <c r="K37" s="33">
         <v>7.79</v>
       </c>
-      <c r="L37" s="31"/>
-      <c r="M37" s="31"/>
-      <c r="N37" s="31"/>
-      <c r="O37" s="31"/>
-      <c r="P37" s="31"/>
-      <c r="Q37" s="31"/>
-      <c r="R37" s="31"/>
-      <c r="S37" s="31"/>
+      <c r="L37" s="32"/>
+      <c r="M37" s="32"/>
+      <c r="N37" s="32"/>
+      <c r="O37" s="32"/>
+      <c r="P37" s="32"/>
+      <c r="Q37" s="32"/>
+      <c r="R37" s="32"/>
+      <c r="S37" s="32"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="27" t="s">
+      <c r="A38" s="28" t="s">
         <v>231</v>
       </c>
-      <c r="B38" s="28"/>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="28"/>
-      <c r="F38" s="28"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="28"/>
-      <c r="I38" s="28"/>
-      <c r="J38" s="28"/>
-      <c r="K38" s="28"/>
-      <c r="L38" s="28"/>
-      <c r="M38" s="28"/>
-      <c r="N38" s="28"/>
-      <c r="O38" s="28"/>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="28"/>
-      <c r="S38" s="28"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="29"/>
+      <c r="F38" s="29"/>
+      <c r="G38" s="29"/>
+      <c r="H38" s="29"/>
+      <c r="I38" s="29"/>
+      <c r="J38" s="29"/>
+      <c r="K38" s="29"/>
+      <c r="L38" s="29"/>
+      <c r="M38" s="29"/>
+      <c r="N38" s="29"/>
+      <c r="O38" s="29"/>
+      <c r="P38" s="29"/>
+      <c r="Q38" s="29"/>
+      <c r="R38" s="29"/>
+      <c r="S38" s="29"/>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="29" t="s">
+      <c r="A39" s="30" t="s">
         <v>232</v>
       </c>
-      <c r="B39" s="32">
+      <c r="B39" s="33">
         <v>46.55</v>
       </c>
-      <c r="C39" s="32">
+      <c r="C39" s="33">
         <v>24.87</v>
       </c>
-      <c r="D39" s="32">
+      <c r="D39" s="33">
         <v>61.02</v>
       </c>
-      <c r="E39" s="32">
+      <c r="E39" s="33">
         <v>28.96</v>
       </c>
-      <c r="F39" s="32">
+      <c r="F39" s="33">
         <v>12.38</v>
       </c>
-      <c r="G39" s="32">
+      <c r="G39" s="33">
         <v>12.51</v>
       </c>
-      <c r="H39" s="32">
+      <c r="H39" s="33">
         <v>26.31</v>
       </c>
-      <c r="I39" s="32">
+      <c r="I39" s="33">
         <v>65.56</v>
       </c>
-      <c r="J39" s="31"/>
-      <c r="K39" s="31"/>
-      <c r="L39" s="31"/>
-      <c r="M39" s="31"/>
-      <c r="N39" s="31"/>
-      <c r="O39" s="31"/>
-      <c r="P39" s="31"/>
-      <c r="Q39" s="31"/>
-      <c r="R39" s="31"/>
-      <c r="S39" s="31"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+      <c r="L39" s="32"/>
+      <c r="M39" s="32"/>
+      <c r="N39" s="32"/>
+      <c r="O39" s="32"/>
+      <c r="P39" s="32"/>
+      <c r="Q39" s="32"/>
+      <c r="R39" s="32"/>
+      <c r="S39" s="32"/>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="29" t="s">
+      <c r="A40" s="30" t="s">
         <v>233</v>
       </c>
-      <c r="B40" s="32">
+      <c r="B40" s="33">
         <v>26.0</v>
       </c>
-      <c r="C40" s="32">
+      <c r="C40" s="33">
         <v>17.15</v>
       </c>
-      <c r="D40" s="32">
+      <c r="D40" s="33">
         <v>18.22</v>
       </c>
-      <c r="E40" s="32">
+      <c r="E40" s="33">
         <v>20.55</v>
       </c>
-      <c r="F40" s="32">
+      <c r="F40" s="33">
         <v>25.61</v>
       </c>
-      <c r="G40" s="32">
+      <c r="G40" s="33">
         <v>48.23</v>
       </c>
-      <c r="H40" s="30">
+      <c r="H40" s="31">
         <v>143.86</v>
       </c>
-      <c r="I40" s="30">
+      <c r="I40" s="31">
         <v>437.51</v>
       </c>
-      <c r="J40" s="31"/>
-      <c r="K40" s="31"/>
-      <c r="L40" s="31"/>
-      <c r="M40" s="31"/>
-      <c r="N40" s="31"/>
-      <c r="O40" s="31"/>
-      <c r="P40" s="31"/>
-      <c r="Q40" s="31"/>
-      <c r="R40" s="31"/>
-      <c r="S40" s="31"/>
+      <c r="J40" s="32"/>
+      <c r="K40" s="32"/>
+      <c r="L40" s="32"/>
+      <c r="M40" s="32"/>
+      <c r="N40" s="32"/>
+      <c r="O40" s="32"/>
+      <c r="P40" s="32"/>
+      <c r="Q40" s="32"/>
+      <c r="R40" s="32"/>
+      <c r="S40" s="32"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="27" t="s">
+      <c r="A41" s="28" t="s">
         <v>234</v>
       </c>
-      <c r="B41" s="28"/>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
-      <c r="E41" s="28"/>
-      <c r="F41" s="28"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="28"/>
-      <c r="I41" s="28"/>
-      <c r="J41" s="28"/>
-      <c r="K41" s="28"/>
-      <c r="L41" s="28"/>
-      <c r="M41" s="28"/>
-      <c r="N41" s="28"/>
-      <c r="O41" s="28"/>
-      <c r="P41" s="28"/>
-      <c r="Q41" s="28"/>
-      <c r="R41" s="28"/>
-      <c r="S41" s="28"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="29"/>
+      <c r="F41" s="29"/>
+      <c r="G41" s="29"/>
+      <c r="H41" s="29"/>
+      <c r="I41" s="29"/>
+      <c r="J41" s="29"/>
+      <c r="K41" s="29"/>
+      <c r="L41" s="29"/>
+      <c r="M41" s="29"/>
+      <c r="N41" s="29"/>
+      <c r="O41" s="29"/>
+      <c r="P41" s="29"/>
+      <c r="Q41" s="29"/>
+      <c r="R41" s="29"/>
+      <c r="S41" s="29"/>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="30" t="s">
         <v>235</v>
       </c>
-      <c r="B42" s="32">
+      <c r="B42" s="33">
         <v>2.72</v>
       </c>
-      <c r="C42" s="32">
+      <c r="C42" s="33">
         <v>2.96</v>
       </c>
-      <c r="D42" s="32">
+      <c r="D42" s="33">
         <v>3.06</v>
       </c>
-      <c r="E42" s="32">
+      <c r="E42" s="33">
         <v>3.03</v>
       </c>
-      <c r="F42" s="32">
+      <c r="F42" s="33">
         <v>2.89</v>
       </c>
-      <c r="G42" s="32">
+      <c r="G42" s="33">
         <v>4.74</v>
       </c>
-      <c r="H42" s="32">
+      <c r="H42" s="33">
         <v>5.23</v>
       </c>
-      <c r="I42" s="32">
+      <c r="I42" s="33">
         <v>5.78</v>
       </c>
-      <c r="J42" s="32">
+      <c r="J42" s="33">
         <v>6.45</v>
       </c>
-      <c r="K42" s="32">
+      <c r="K42" s="33">
         <v>7.79</v>
       </c>
-      <c r="L42" s="31"/>
-      <c r="M42" s="31"/>
-      <c r="N42" s="31"/>
-      <c r="O42" s="31"/>
-      <c r="P42" s="31"/>
-      <c r="Q42" s="31"/>
-      <c r="R42" s="31"/>
-      <c r="S42" s="31"/>
+      <c r="L42" s="32"/>
+      <c r="M42" s="32"/>
+      <c r="N42" s="32"/>
+      <c r="O42" s="32"/>
+      <c r="P42" s="32"/>
+      <c r="Q42" s="32"/>
+      <c r="R42" s="32"/>
+      <c r="S42" s="32"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="28" t="s">
         <v>236</v>
       </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="28"/>
-      <c r="L43" s="28"/>
-      <c r="M43" s="28"/>
-      <c r="N43" s="28"/>
-      <c r="O43" s="28"/>
-      <c r="P43" s="28"/>
-      <c r="Q43" s="28"/>
-      <c r="R43" s="28"/>
-      <c r="S43" s="28"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
+      <c r="L43" s="29"/>
+      <c r="M43" s="29"/>
+      <c r="N43" s="29"/>
+      <c r="O43" s="29"/>
+      <c r="P43" s="29"/>
+      <c r="Q43" s="29"/>
+      <c r="R43" s="29"/>
+      <c r="S43" s="29"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="29" t="s">
+      <c r="A44" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="B44" s="32">
+      <c r="B44" s="33">
         <v>49.47</v>
       </c>
-      <c r="C44" s="32">
+      <c r="C44" s="33">
         <v>25.04</v>
       </c>
-      <c r="D44" s="32">
+      <c r="D44" s="33">
         <v>61.88</v>
       </c>
-      <c r="E44" s="32">
+      <c r="E44" s="33">
         <v>25.31</v>
       </c>
-      <c r="F44" s="32">
+      <c r="F44" s="33">
         <v>23.36</v>
       </c>
-      <c r="G44" s="32">
+      <c r="G44" s="33">
         <v>9.88</v>
       </c>
-      <c r="H44" s="32">
+      <c r="H44" s="33">
         <v>18.16</v>
       </c>
-      <c r="I44" s="32">
+      <c r="I44" s="33">
         <v>42.77</v>
       </c>
-      <c r="J44" s="31"/>
-      <c r="K44" s="31"/>
-      <c r="L44" s="31"/>
-      <c r="M44" s="31"/>
-      <c r="N44" s="31"/>
-      <c r="O44" s="31"/>
-      <c r="P44" s="31"/>
-      <c r="Q44" s="31"/>
-      <c r="R44" s="31"/>
-      <c r="S44" s="31"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="32"/>
+      <c r="L44" s="32"/>
+      <c r="M44" s="32"/>
+      <c r="N44" s="32"/>
+      <c r="O44" s="32"/>
+      <c r="P44" s="32"/>
+      <c r="Q44" s="32"/>
+      <c r="R44" s="32"/>
+      <c r="S44" s="32"/>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="29" t="s">
+      <c r="A45" s="30" t="s">
         <v>238</v>
       </c>
-      <c r="B45" s="32">
+      <c r="B45" s="33">
         <v>34.3</v>
       </c>
-      <c r="C45" s="32">
+      <c r="C45" s="33">
         <v>23.07</v>
       </c>
-      <c r="D45" s="32">
+      <c r="D45" s="33">
         <v>21.88</v>
       </c>
-      <c r="E45" s="32">
+      <c r="E45" s="33">
         <v>18.83</v>
       </c>
-      <c r="F45" s="32">
+      <c r="F45" s="33">
         <v>20.1</v>
       </c>
-      <c r="G45" s="32">
+      <c r="G45" s="33">
         <v>29.47</v>
       </c>
-      <c r="H45" s="32">
+      <c r="H45" s="33">
         <v>82.73</v>
       </c>
-      <c r="I45" s="30">
+      <c r="I45" s="31">
         <v>237.07</v>
       </c>
-      <c r="J45" s="31"/>
-      <c r="K45" s="31"/>
-      <c r="L45" s="31"/>
-      <c r="M45" s="31"/>
-      <c r="N45" s="31"/>
-      <c r="O45" s="31"/>
-      <c r="P45" s="31"/>
-      <c r="Q45" s="31"/>
-      <c r="R45" s="31"/>
-      <c r="S45" s="31"/>
+      <c r="J45" s="32"/>
+      <c r="K45" s="32"/>
+      <c r="L45" s="32"/>
+      <c r="M45" s="32"/>
+      <c r="N45" s="32"/>
+      <c r="O45" s="32"/>
+      <c r="P45" s="32"/>
+      <c r="Q45" s="32"/>
+      <c r="R45" s="32"/>
+      <c r="S45" s="32"/>
     </row>
     <row r="46" ht="15.75" customHeight="1"/>
     <row r="47" ht="15.75" customHeight="1"/>
@@ -11189,19 +11225,19 @@
         <v>242</v>
       </c>
       <c r="B20" s="16"/>
-      <c r="C20" s="26">
+      <c r="C20" s="27">
         <v>-321.98</v>
       </c>
-      <c r="D20" s="26">
+      <c r="D20" s="27">
         <v>-307.84</v>
       </c>
-      <c r="E20" s="26">
+      <c r="E20" s="27">
         <v>-175.21</v>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="27">
         <v>-102.08</v>
       </c>
-      <c r="G20" s="26">
+      <c r="G20" s="27">
         <v>-180.84</v>
       </c>
       <c r="H20" s="16"/>
@@ -11334,22 +11370,22 @@
       <c r="A25" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="B25" s="26">
+      <c r="B25" s="27">
         <v>-362.34</v>
       </c>
-      <c r="C25" s="26">
+      <c r="C25" s="27">
         <v>-349.03</v>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="27">
         <v>-325.26</v>
       </c>
-      <c r="E25" s="26">
+      <c r="E25" s="27">
         <v>-184.14</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="27">
         <v>-104.77</v>
       </c>
-      <c r="G25" s="26">
+      <c r="G25" s="27">
         <v>-183.33</v>
       </c>
       <c r="H25" s="21">
@@ -11487,7 +11523,7 @@
       </c>
       <c r="I30" s="16"/>
       <c r="J30" s="16"/>
-      <c r="K30" s="23">
+      <c r="K30" s="24">
         <v>0.0</v>
       </c>
       <c r="L30" s="21">
@@ -11552,7 +11588,7 @@
       <c r="E33" s="16"/>
       <c r="F33" s="16"/>
       <c r="G33" s="16"/>
-      <c r="H33" s="23">
+      <c r="H33" s="24">
         <v>0.0</v>
       </c>
       <c r="I33" s="16"/>
@@ -11566,37 +11602,37 @@
       <c r="A34" s="17" t="s">
         <v>254</v>
       </c>
-      <c r="B34" s="24">
+      <c r="B34" s="25">
         <v>-282.8</v>
       </c>
-      <c r="C34" s="24">
+      <c r="C34" s="25">
         <v>-231.77</v>
       </c>
-      <c r="D34" s="24">
+      <c r="D34" s="25">
         <v>-277.08</v>
       </c>
-      <c r="E34" s="24">
+      <c r="E34" s="25">
         <v>-164.85</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="25">
         <v>-130.4</v>
       </c>
-      <c r="G34" s="24">
+      <c r="G34" s="25">
         <v>-137.8</v>
       </c>
-      <c r="H34" s="25">
+      <c r="H34" s="26">
         <v>-58.29</v>
       </c>
-      <c r="I34" s="25">
+      <c r="I34" s="26">
         <v>-76.8</v>
       </c>
-      <c r="J34" s="25">
+      <c r="J34" s="26">
         <v>-83.81</v>
       </c>
-      <c r="K34" s="25">
+      <c r="K34" s="26">
         <v>-35.46</v>
       </c>
-      <c r="L34" s="25">
+      <c r="L34" s="26">
         <v>-48.91</v>
       </c>
     </row>
@@ -11698,22 +11734,22 @@
       <c r="A39" s="17" t="s">
         <v>259</v>
       </c>
-      <c r="B39" s="25">
+      <c r="B39" s="26">
         <v>-2.97</v>
       </c>
-      <c r="C39" s="25">
+      <c r="C39" s="26">
         <v>-1.22</v>
       </c>
       <c r="D39" s="19">
         <v>0.0</v>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="26">
         <v>-1.62</v>
       </c>
-      <c r="F39" s="25">
+      <c r="F39" s="26">
         <v>-5.97</v>
       </c>
-      <c r="G39" s="25">
+      <c r="G39" s="26">
         <v>-60.94</v>
       </c>
       <c r="H39" s="19"/>
@@ -11930,22 +11966,22 @@
       <c r="A47" s="17" t="s">
         <v>267</v>
       </c>
-      <c r="B47" s="22">
+      <c r="B47" s="23">
         <v>148.28</v>
       </c>
-      <c r="C47" s="22">
+      <c r="C47" s="23">
         <v>275.5</v>
       </c>
-      <c r="D47" s="22">
+      <c r="D47" s="23">
         <v>456.73</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E47" s="23">
         <v>147.94</v>
       </c>
-      <c r="F47" s="25">
+      <c r="F47" s="26">
         <v>-8.92</v>
       </c>
-      <c r="G47" s="22">
+      <c r="G47" s="23">
         <v>233.77</v>
       </c>
       <c r="H47" s="18">
@@ -11957,7 +11993,7 @@
       <c r="J47" s="18">
         <v>2.02</v>
       </c>
-      <c r="K47" s="22">
+      <c r="K47" s="23">
         <v>372.9</v>
       </c>
       <c r="L47" s="18">
@@ -12044,7 +12080,7 @@
       <c r="A50" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="B50" s="26">
+      <c r="B50" s="27">
         <v>-137.48</v>
       </c>
       <c r="C50" s="15">
@@ -12056,7 +12092,7 @@
       <c r="E50" s="21">
         <v>-18.53</v>
       </c>
-      <c r="F50" s="26">
+      <c r="F50" s="27">
         <v>-145.29</v>
       </c>
       <c r="G50" s="15">
@@ -12108,19 +12144,19 @@
       <c r="A52" s="17" t="s">
         <v>272</v>
       </c>
-      <c r="B52" s="24">
+      <c r="B52" s="25">
         <v>-143.2</v>
       </c>
       <c r="C52" s="18">
         <v>48.41</v>
       </c>
-      <c r="D52" s="22">
+      <c r="D52" s="23">
         <v>174.87</v>
       </c>
-      <c r="E52" s="25">
+      <c r="E52" s="26">
         <v>-15.49</v>
       </c>
-      <c r="F52" s="24">
+      <c r="F52" s="25">
         <v>-144.2</v>
       </c>
       <c r="G52" s="18">
@@ -12129,16 +12165,16 @@
       <c r="H52" s="18">
         <v>23.47</v>
       </c>
-      <c r="I52" s="25">
+      <c r="I52" s="26">
         <v>-74.59</v>
       </c>
-      <c r="J52" s="25">
+      <c r="J52" s="26">
         <v>-81.79</v>
       </c>
-      <c r="K52" s="22">
+      <c r="K52" s="23">
         <v>337.44</v>
       </c>
-      <c r="L52" s="25">
+      <c r="L52" s="26">
         <v>-47.75</v>
       </c>
     </row>
@@ -12191,10 +12227,10 @@
       <c r="F54" s="21">
         <v>-0.04</v>
       </c>
-      <c r="G54" s="23">
-        <v>0.0</v>
-      </c>
-      <c r="H54" s="23">
+      <c r="G54" s="24">
+        <v>0.0</v>
+      </c>
+      <c r="H54" s="24">
         <v>0.0</v>
       </c>
       <c r="I54" s="16"/>

</xml_diff>